<commit_message>
Force automatic full calculation mode in the workbook
Fixes portfolio/total tax showing $0 after editing inputs in Excel: the
file didn't explicitly set calcMode, so it could inherit a Manual
calculation setting from the user's Excel app, leaving long formula
chains (the hidden bracket-tax engine) stale until a manual recalc.
Explicitly setting calcMode=auto + forceFullCalc ensures the workbook
always recalculates automatically regardless of the app's prior setting.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XveA8LngnD1MFNqnzekQW3
</commit_message>
<xml_diff>
--- a/Tax_Estimator_and_Portfolio_Tax_Calculator.xlsx
+++ b/Tax_Estimator_and_Portfolio_Tax_Calculator.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Tax Information" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -914,7 +914,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N147"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
@@ -952,12 +952,6 @@
           <t>STEP 1 - YOUR INFORMATION</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="21" t="inlineStr">
@@ -1031,8 +1025,6 @@
           <t>YOUR STATE TAX RATE</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="24" t="inlineStr">
@@ -1083,12 +1075,6 @@
           <t>STEP 2 - INCOME</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr"/>
@@ -1218,12 +1204,6 @@
           <t>PRE-TAX CONTRIBUTIONS</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="5" t="inlineStr"/>
@@ -1296,12 +1276,6 @@
           <t>DEDUCTIONS</t>
         </is>
       </c>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="21" t="inlineStr">
@@ -1361,12 +1335,6 @@
           <t>STEP 3 - YOUR ESTIMATED TAX</t>
         </is>
       </c>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="B46" s="29" t="inlineStr">
@@ -1414,7 +1382,6 @@
           <t>Tax Breakdown</t>
         </is>
       </c>
-      <c r="C49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="B50" s="24" t="inlineStr">
@@ -2657,8 +2624,8 @@
     <mergeCell ref="B79:E79"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="C15:D15"/>
-    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="A2:G2"/>
@@ -2736,12 +2703,6 @@
           <t>YOUR INFORMATION</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="21" t="inlineStr">
@@ -2793,8 +2754,6 @@
           <t>YOUR STATE TAX RATE</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="24" t="inlineStr">
@@ -2838,12 +2797,6 @@
           <t>INCOME (used to determine your tax bracket)</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="24" t="inlineStr">
@@ -2871,12 +2824,6 @@
           <t>PORTFOLIO INCOME</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="24" t="inlineStr">
@@ -2974,12 +2921,6 @@
           <t>YOUR PORTFOLIO TAX</t>
         </is>
       </c>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="29" t="inlineStr">
@@ -3027,7 +2968,6 @@
           <t>Portfolio Tax Estimate</t>
         </is>
       </c>
-      <c r="C34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="24" t="inlineStr">
@@ -3112,7 +3052,6 @@
           <t>Tax by Income Type</t>
         </is>
       </c>
-      <c r="C43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="F44" s="7" t="inlineStr">
@@ -4131,7 +4070,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA208"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -4181,29 +4120,6 @@
           <t>Federal Ordinary Income Tax Brackets</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="4" t="n"/>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="4" t="n"/>
-      <c r="R4" s="4" t="n"/>
-      <c r="S4" s="4" t="n"/>
-      <c r="T4" s="4" t="n"/>
-      <c r="U4" s="4" t="n"/>
-      <c r="V4" s="4" t="n"/>
-      <c r="W4" s="4" t="n"/>
-      <c r="X4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -5163,29 +5079,6 @@
           <t>Long-Term Capital Gains / Qualified Dividend Brackets (0% / 15% / 20%)</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="n"/>
-      <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="n"/>
-      <c r="K17" s="4" t="n"/>
-      <c r="L17" s="4" t="n"/>
-      <c r="M17" s="4" t="n"/>
-      <c r="N17" s="4" t="n"/>
-      <c r="O17" s="4" t="n"/>
-      <c r="P17" s="4" t="n"/>
-      <c r="Q17" s="4" t="n"/>
-      <c r="R17" s="4" t="n"/>
-      <c r="S17" s="4" t="n"/>
-      <c r="T17" s="4" t="n"/>
-      <c r="U17" s="4" t="n"/>
-      <c r="V17" s="4" t="n"/>
-      <c r="W17" s="4" t="n"/>
-      <c r="X17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -5685,29 +5578,6 @@
           <t>Standard Deduction</t>
         </is>
       </c>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
-      <c r="H30" s="4" t="n"/>
-      <c r="I30" s="4" t="n"/>
-      <c r="J30" s="4" t="n"/>
-      <c r="K30" s="4" t="n"/>
-      <c r="L30" s="4" t="n"/>
-      <c r="M30" s="4" t="n"/>
-      <c r="N30" s="4" t="n"/>
-      <c r="O30" s="4" t="n"/>
-      <c r="P30" s="4" t="n"/>
-      <c r="Q30" s="4" t="n"/>
-      <c r="R30" s="4" t="n"/>
-      <c r="S30" s="4" t="n"/>
-      <c r="T30" s="4" t="n"/>
-      <c r="U30" s="4" t="n"/>
-      <c r="V30" s="4" t="n"/>
-      <c r="W30" s="4" t="n"/>
-      <c r="X30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -5907,29 +5777,6 @@
           <t>NIIT, Additional Medicare Tax &amp; Capital-Loss Thresholds (fixed by statute)</t>
         </is>
       </c>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
-      <c r="H43" s="4" t="n"/>
-      <c r="I43" s="4" t="n"/>
-      <c r="J43" s="4" t="n"/>
-      <c r="K43" s="4" t="n"/>
-      <c r="L43" s="4" t="n"/>
-      <c r="M43" s="4" t="n"/>
-      <c r="N43" s="4" t="n"/>
-      <c r="O43" s="4" t="n"/>
-      <c r="P43" s="4" t="n"/>
-      <c r="Q43" s="4" t="n"/>
-      <c r="R43" s="4" t="n"/>
-      <c r="S43" s="4" t="n"/>
-      <c r="T43" s="4" t="n"/>
-      <c r="U43" s="4" t="n"/>
-      <c r="V43" s="4" t="n"/>
-      <c r="W43" s="4" t="n"/>
-      <c r="X43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -6039,29 +5886,6 @@
           <t>SALT (State &amp; Local Tax) Itemized Deduction Cap</t>
         </is>
       </c>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
-      <c r="J51" s="4" t="n"/>
-      <c r="K51" s="4" t="n"/>
-      <c r="L51" s="4" t="n"/>
-      <c r="M51" s="4" t="n"/>
-      <c r="N51" s="4" t="n"/>
-      <c r="O51" s="4" t="n"/>
-      <c r="P51" s="4" t="n"/>
-      <c r="Q51" s="4" t="n"/>
-      <c r="R51" s="4" t="n"/>
-      <c r="S51" s="4" t="n"/>
-      <c r="T51" s="4" t="n"/>
-      <c r="U51" s="4" t="n"/>
-      <c r="V51" s="4" t="n"/>
-      <c r="W51" s="4" t="n"/>
-      <c r="X51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -6261,29 +6085,6 @@
           <t>Payroll (FICA) &amp; Self-Employment Tax Parameters</t>
         </is>
       </c>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="4" t="n"/>
-      <c r="E64" s="4" t="n"/>
-      <c r="F64" s="4" t="n"/>
-      <c r="G64" s="4" t="n"/>
-      <c r="H64" s="4" t="n"/>
-      <c r="I64" s="4" t="n"/>
-      <c r="J64" s="4" t="n"/>
-      <c r="K64" s="4" t="n"/>
-      <c r="L64" s="4" t="n"/>
-      <c r="M64" s="4" t="n"/>
-      <c r="N64" s="4" t="n"/>
-      <c r="O64" s="4" t="n"/>
-      <c r="P64" s="4" t="n"/>
-      <c r="Q64" s="4" t="n"/>
-      <c r="R64" s="4" t="n"/>
-      <c r="S64" s="4" t="n"/>
-      <c r="T64" s="4" t="n"/>
-      <c r="U64" s="4" t="n"/>
-      <c r="V64" s="4" t="n"/>
-      <c r="W64" s="4" t="n"/>
-      <c r="X64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -6396,29 +6197,6 @@
           <t>State Master List &amp; Income Treatment</t>
         </is>
       </c>
-      <c r="B69" s="4" t="n"/>
-      <c r="C69" s="4" t="n"/>
-      <c r="D69" s="4" t="n"/>
-      <c r="E69" s="4" t="n"/>
-      <c r="F69" s="4" t="n"/>
-      <c r="G69" s="4" t="n"/>
-      <c r="H69" s="4" t="n"/>
-      <c r="I69" s="4" t="n"/>
-      <c r="J69" s="4" t="n"/>
-      <c r="K69" s="4" t="n"/>
-      <c r="L69" s="4" t="n"/>
-      <c r="M69" s="4" t="n"/>
-      <c r="N69" s="4" t="n"/>
-      <c r="O69" s="4" t="n"/>
-      <c r="P69" s="4" t="n"/>
-      <c r="Q69" s="4" t="n"/>
-      <c r="R69" s="4" t="n"/>
-      <c r="S69" s="4" t="n"/>
-      <c r="T69" s="4" t="n"/>
-      <c r="U69" s="4" t="n"/>
-      <c r="V69" s="4" t="n"/>
-      <c r="W69" s="4" t="n"/>
-      <c r="X69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -7684,29 +7462,6 @@
           <t>State Income Tax Brackets (unified format; category Single covers Single/MFS/HOH, MFJ covers MFJ/QSS)</t>
         </is>
       </c>
-      <c r="B104" s="4" t="n"/>
-      <c r="C104" s="4" t="n"/>
-      <c r="D104" s="4" t="n"/>
-      <c r="E104" s="4" t="n"/>
-      <c r="F104" s="4" t="n"/>
-      <c r="G104" s="4" t="n"/>
-      <c r="H104" s="4" t="n"/>
-      <c r="I104" s="4" t="n"/>
-      <c r="J104" s="4" t="n"/>
-      <c r="K104" s="4" t="n"/>
-      <c r="L104" s="4" t="n"/>
-      <c r="M104" s="4" t="n"/>
-      <c r="N104" s="4" t="n"/>
-      <c r="O104" s="4" t="n"/>
-      <c r="P104" s="4" t="n"/>
-      <c r="Q104" s="4" t="n"/>
-      <c r="R104" s="4" t="n"/>
-      <c r="S104" s="4" t="n"/>
-      <c r="T104" s="4" t="n"/>
-      <c r="U104" s="4" t="n"/>
-      <c r="V104" s="4" t="n"/>
-      <c r="W104" s="4" t="n"/>
-      <c r="X104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
@@ -13931,29 +13686,6 @@
           <t>Local / Municipal Tax Table</t>
         </is>
       </c>
-      <c r="B171" s="4" t="n"/>
-      <c r="C171" s="4" t="n"/>
-      <c r="D171" s="4" t="n"/>
-      <c r="E171" s="4" t="n"/>
-      <c r="F171" s="4" t="n"/>
-      <c r="G171" s="4" t="n"/>
-      <c r="H171" s="4" t="n"/>
-      <c r="I171" s="4" t="n"/>
-      <c r="J171" s="4" t="n"/>
-      <c r="K171" s="4" t="n"/>
-      <c r="L171" s="4" t="n"/>
-      <c r="M171" s="4" t="n"/>
-      <c r="N171" s="4" t="n"/>
-      <c r="O171" s="4" t="n"/>
-      <c r="P171" s="4" t="n"/>
-      <c r="Q171" s="4" t="n"/>
-      <c r="R171" s="4" t="n"/>
-      <c r="S171" s="4" t="n"/>
-      <c r="T171" s="4" t="n"/>
-      <c r="U171" s="4" t="n"/>
-      <c r="V171" s="4" t="n"/>
-      <c r="W171" s="4" t="n"/>
-      <c r="X171" s="4" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="5" t="inlineStr">
@@ -14405,93 +14137,17 @@
           <t>DISCLAIMER: Tax estimates are for educational and financial-planning purposes only. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. This calculator does not provide tax, legal, or accounting advice. Consult a qualified tax professional regarding your individual situation.</t>
         </is>
       </c>
-      <c r="B189" s="17" t="n"/>
-      <c r="C189" s="17" t="n"/>
-      <c r="D189" s="17" t="n"/>
-      <c r="E189" s="17" t="n"/>
-      <c r="F189" s="17" t="n"/>
-      <c r="G189" s="17" t="n"/>
-      <c r="H189" s="17" t="n"/>
-      <c r="I189" s="17" t="n"/>
-      <c r="J189" s="17" t="n"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="17" t="n"/>
-      <c r="B190" s="17" t="n"/>
-      <c r="C190" s="17" t="n"/>
-      <c r="D190" s="17" t="n"/>
-      <c r="E190" s="17" t="n"/>
-      <c r="F190" s="17" t="n"/>
-      <c r="G190" s="17" t="n"/>
-      <c r="H190" s="17" t="n"/>
-      <c r="I190" s="17" t="n"/>
-      <c r="J190" s="17" t="n"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="17" t="n"/>
-      <c r="B191" s="17" t="n"/>
-      <c r="C191" s="17" t="n"/>
-      <c r="D191" s="17" t="n"/>
-      <c r="E191" s="17" t="n"/>
-      <c r="F191" s="17" t="n"/>
-      <c r="G191" s="17" t="n"/>
-      <c r="H191" s="17" t="n"/>
-      <c r="I191" s="17" t="n"/>
-      <c r="J191" s="17" t="n"/>
-    </row>
-    <row r="192">
-      <c r="A192" s="17" t="n"/>
-      <c r="B192" s="17" t="n"/>
-      <c r="C192" s="17" t="n"/>
-      <c r="D192" s="17" t="n"/>
-      <c r="E192" s="17" t="n"/>
-      <c r="F192" s="17" t="n"/>
-      <c r="G192" s="17" t="n"/>
-      <c r="H192" s="17" t="n"/>
-      <c r="I192" s="17" t="n"/>
-      <c r="J192" s="17" t="n"/>
-    </row>
-    <row r="193">
-      <c r="A193" s="17" t="n"/>
-      <c r="B193" s="17" t="n"/>
-      <c r="C193" s="17" t="n"/>
-      <c r="D193" s="17" t="n"/>
-      <c r="E193" s="17" t="n"/>
-      <c r="F193" s="17" t="n"/>
-      <c r="G193" s="17" t="n"/>
-      <c r="H193" s="17" t="n"/>
-      <c r="I193" s="17" t="n"/>
-      <c r="J193" s="17" t="n"/>
-    </row>
+    </row>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
     <row r="195" ht="18" customHeight="1">
       <c r="A195" s="3" t="inlineStr">
         <is>
           <t>Key Assumptions</t>
         </is>
       </c>
-      <c r="B195" s="4" t="n"/>
-      <c r="C195" s="4" t="n"/>
-      <c r="D195" s="4" t="n"/>
-      <c r="E195" s="4" t="n"/>
-      <c r="F195" s="4" t="n"/>
-      <c r="G195" s="4" t="n"/>
-      <c r="H195" s="4" t="n"/>
-      <c r="I195" s="4" t="n"/>
-      <c r="J195" s="4" t="n"/>
-      <c r="K195" s="4" t="n"/>
-      <c r="L195" s="4" t="n"/>
-      <c r="M195" s="4" t="n"/>
-      <c r="N195" s="4" t="n"/>
-      <c r="O195" s="4" t="n"/>
-      <c r="P195" s="4" t="n"/>
-      <c r="Q195" s="4" t="n"/>
-      <c r="R195" s="4" t="n"/>
-      <c r="S195" s="4" t="n"/>
-      <c r="T195" s="4" t="n"/>
-      <c r="U195" s="4" t="n"/>
-      <c r="V195" s="4" t="n"/>
-      <c r="W195" s="4" t="n"/>
-      <c r="X195" s="4" t="n"/>
     </row>
     <row r="196" ht="40" customHeight="1">
       <c r="A196" s="18" t="inlineStr">

</xml_diff>